<commit_message>
feat: add data files
</commit_message>
<xml_diff>
--- a/для бд nosologies.xlsx
+++ b/для бд nosologies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\easymed-analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7E5249-59A7-462F-BD88-4391285D36F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDFBED04-AD60-4DD8-B100-73E19D0F0690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6AA829BB-BB4D-4D68-9527-FAF90550C0CB}"/>
   </bookViews>
@@ -164,898 +164,898 @@
     <t>T33-T35</t>
   </si>
   <si>
-    <t>Термические и химические ожоги  (3)</t>
-  </si>
-  <si>
     <t>T20-T32</t>
   </si>
   <si>
-    <t>Последствия проникновения инородного тела через естественные отверстия  (2)</t>
-  </si>
-  <si>
     <t>T15-T19</t>
   </si>
   <si>
-    <t>Травмы неуточненной части туловища, конечности или области тела  (1)</t>
-  </si>
-  <si>
     <t>T08-T14</t>
   </si>
   <si>
-    <t>Травмы, захватывающие несколько областей тела  (4)</t>
-  </si>
-  <si>
     <t>T00-T07</t>
   </si>
   <si>
-    <t>Травмы области голеностопного сустава и стопы  (4)</t>
-  </si>
-  <si>
     <t>S90-S99</t>
   </si>
   <si>
-    <t>Травмы колена и голени  (11)</t>
-  </si>
-  <si>
     <t>S80-S89</t>
   </si>
   <si>
-    <t>Травмы области тазобедренного сустава и бедра  (3)</t>
-  </si>
-  <si>
     <t>S70-S79</t>
   </si>
   <si>
-    <t>Травмы запястья и кисти  (3)</t>
-  </si>
-  <si>
     <t>S60-S69</t>
   </si>
   <si>
-    <t>Травмы локтя и предплечья  (4)</t>
-  </si>
-  <si>
     <t>S50-S59</t>
   </si>
   <si>
-    <t>Травмы плечевого пояса и плеча  (5)</t>
-  </si>
-  <si>
     <t>S40-S49</t>
   </si>
   <si>
-    <t>Травмы живота, нижней части спины, поясничного отдела позвоночника и таза  (3)</t>
-  </si>
-  <si>
     <t>S30-S39</t>
   </si>
   <si>
-    <t>Травмы грудной клетки  (2)</t>
-  </si>
-  <si>
     <t>S20-S29</t>
   </si>
   <si>
-    <t>Травмы шеи  (2)</t>
-  </si>
-  <si>
     <t>S10-S19</t>
   </si>
   <si>
-    <t>Травмы головы  (13)</t>
-  </si>
-  <si>
     <t>S00-S09</t>
   </si>
   <si>
-    <t>Отклонения от нормы, выявленные при исследовании крови, при отсутствии установленного диагноза  (3)</t>
-  </si>
-  <si>
     <t>R70-R79</t>
   </si>
   <si>
-    <t>Общие симптомы и признаки  (3)</t>
-  </si>
-  <si>
     <t>R50-R69</t>
   </si>
   <si>
-    <t>Симптомы и признаки, относящиеся к мочевой системе  (1)</t>
-  </si>
-  <si>
     <t>R30-R39</t>
   </si>
   <si>
-    <t>Симптомы и признаки, относящиеся к системе пищеварения и брюшной полости  (2)</t>
-  </si>
-  <si>
     <t>R10-R19</t>
   </si>
   <si>
-    <t>Другие болезни, вызываемые хламидиями  (1)</t>
-  </si>
-  <si>
     <t>A70-A74</t>
   </si>
   <si>
-    <t>Вирусные инфекции центральной нервной системы  (1)</t>
-  </si>
-  <si>
     <t>A80-A89</t>
   </si>
   <si>
-    <t>Вирусные лихорадки, передаваемые членистоногими, и вирусные геморрагические лихорадки  (2)</t>
-  </si>
-  <si>
     <t>A90-A99</t>
   </si>
   <si>
-    <t>Вирусные инфекции, характеризующиеся поражениями кожи и слизистых оболочек  (5)</t>
-  </si>
-  <si>
     <t>B00-B09</t>
   </si>
   <si>
-    <t>Вирусный гепатит  (6)</t>
-  </si>
-  <si>
     <t>B15-B19</t>
   </si>
   <si>
-    <t>Болезнь, вызванная вирусом иммунодефицита человека [вич]  (3)</t>
-  </si>
-  <si>
     <t>B20-B24</t>
   </si>
   <si>
-    <t>Другие вирусные болезни  (3)</t>
-  </si>
-  <si>
     <t>B25-B34</t>
   </si>
   <si>
-    <t>Микозы  (4)</t>
-  </si>
-  <si>
     <t>B35-B49</t>
   </si>
   <si>
-    <t>Гельминтозы  (2)</t>
-  </si>
-  <si>
     <t>B65-B83</t>
   </si>
   <si>
-    <t>Последствия инфекционных и паразитарных болезней  (1)</t>
-  </si>
-  <si>
     <t>B90-B94</t>
   </si>
   <si>
-    <t>Бактериальные, вирусные и другие инфекционные агенты  (2)</t>
-  </si>
-  <si>
     <t>B95-B97</t>
   </si>
   <si>
-    <t>Злокачественные новообразования  (74)</t>
-  </si>
-  <si>
     <t>C00-C97</t>
   </si>
   <si>
-    <t>Новообразования in situ  (9)</t>
-  </si>
-  <si>
     <t>D00-D09</t>
   </si>
   <si>
-    <t>Доброкачественные новообразования  (11)</t>
-  </si>
-  <si>
     <t>D10-D36</t>
   </si>
   <si>
-    <t>Новообразования неопределенного или неизвестного характера  (21)</t>
-  </si>
-  <si>
     <t>D37-D48</t>
   </si>
   <si>
-    <t>Анемии, связанные с питанием  (3)</t>
-  </si>
-  <si>
     <t>D50-D53</t>
   </si>
   <si>
-    <t>Гемолитические анемии  (4)</t>
-  </si>
-  <si>
     <t>D55-D59</t>
   </si>
   <si>
-    <t>Апластические и другие анемии  (6)</t>
-  </si>
-  <si>
     <t>D60-D64</t>
   </si>
   <si>
-    <t>Нарушения свертываемости крови, пурпура и другие геморрагические состояния  (3)</t>
-  </si>
-  <si>
     <t>D65-D69</t>
   </si>
   <si>
-    <t>Другие болезни крови и кроветворных органов  (1)</t>
-  </si>
-  <si>
     <t>D70-D77</t>
   </si>
   <si>
-    <t>Отдельные нарушения, вовлекающие иммунный механизм  (3)</t>
-  </si>
-  <si>
     <t>D80-D89</t>
   </si>
   <si>
-    <t>Другие врожденные аномалии [пороки развития]  (2)</t>
-  </si>
-  <si>
     <t>Q80-Q89</t>
   </si>
   <si>
-    <t>Симптомы и признаки, относящиеся к системам кровообращения и дыхания  (1)</t>
-  </si>
-  <si>
     <t>R00-R09</t>
   </si>
   <si>
-    <t>Врожденные аномалии [пороки развития] и деформации костно-мышечной системы  (2)</t>
-  </si>
-  <si>
     <t>Q65-Q79</t>
   </si>
   <si>
-    <t>Врожденные аномалии [пороки развития] мочевой системы  (2)</t>
-  </si>
-  <si>
     <t>Q60-Q64</t>
   </si>
   <si>
-    <t>Другие врожденные аномалии [пороки развития] органов пищеварения  (1)</t>
-  </si>
-  <si>
     <t>Q38-Q45</t>
   </si>
   <si>
-    <t>Врожденные аномалии [пороки развития] системы кровообращения  (19)</t>
-  </si>
-  <si>
     <t>Q20-Q28</t>
   </si>
   <si>
-    <t>Врожденные аномалии [пороки развития] глаза, уха, лица и шеи  (2)</t>
-  </si>
-  <si>
     <t>Q10-Q18</t>
   </si>
   <si>
-    <t>Другие нарушения, возникающие в перинатальном периоде  (1)</t>
-  </si>
-  <si>
     <t>P90-P96</t>
   </si>
   <si>
-    <t>Геморрагические и гематологические нарушения у плода и новорожденного  (1)</t>
-  </si>
-  <si>
     <t>P50-P61</t>
   </si>
   <si>
-    <t>Инфекционные болезни, специфичные для перинатального периода  (2)</t>
-  </si>
-  <si>
     <t>P35-P39</t>
   </si>
   <si>
-    <t>Дыхательные и сердечно-сосудистые нарушения, характерные для перинатального периода  (1)</t>
-  </si>
-  <si>
     <t>P20-P29</t>
   </si>
   <si>
-    <t>Расстройства, связанные с продолжительностью беременности и ростом плода  (1)</t>
-  </si>
-  <si>
     <t>P05-P08</t>
   </si>
   <si>
-    <t>Другие акушерские состояния, не классифицированные в других рубриках  (3)</t>
-  </si>
-  <si>
     <t>O95-O99</t>
   </si>
   <si>
-    <t>Болезни щитовидной железы  (5)</t>
-  </si>
-  <si>
     <t>E00-E07</t>
   </si>
   <si>
-    <t>Сахарный диабет  (4)</t>
-  </si>
-  <si>
     <t>E10-E14</t>
   </si>
   <si>
-    <t>Нарушения других эндокринных желез  (7)</t>
-  </si>
-  <si>
     <t>E20-E35</t>
   </si>
   <si>
-    <t>Недостаточность питания  (2)</t>
-  </si>
-  <si>
     <t>E40-E46</t>
   </si>
   <si>
-    <t>Другие виды недостаточности питания  (2)</t>
-  </si>
-  <si>
     <t>E50-E64</t>
   </si>
   <si>
-    <t>Ожирение и другие виды избыточности питания  (1)</t>
-  </si>
-  <si>
     <t>E65-E68</t>
   </si>
   <si>
-    <t>Нарушения обмена веществ  (29)</t>
-  </si>
-  <si>
     <t>E70-E90</t>
   </si>
   <si>
-    <t>Органические, включая симптоматические, психические расстройства  (4)</t>
-  </si>
-  <si>
     <t>F00-F09</t>
   </si>
   <si>
-    <t>Психические расстройства и расстройства поведения, связанные с употреблением психоактивных веществ  (10)</t>
-  </si>
-  <si>
     <t>F10-F19</t>
   </si>
   <si>
-    <t>Шизофрения, шизотипические состояния и бредовые расстройства  (1)</t>
-  </si>
-  <si>
     <t>F20-F29</t>
   </si>
   <si>
-    <t>Расстройства настроения [аффективные расстройства]  (2)</t>
-  </si>
-  <si>
     <t>F30-F39</t>
   </si>
   <si>
-    <t>Невротические, связанные со стрессом и соматоформные расстройства  (5)</t>
-  </si>
-  <si>
     <t>F40-F48</t>
   </si>
   <si>
-    <t>Поведенческие синдромы, связанные с физиологическими нарушениями и физическими факторами  (1)</t>
-  </si>
-  <si>
     <t>F50-F59</t>
   </si>
   <si>
-    <t>Расстройства личности и поведения в зрелом возрасте  (1)</t>
-  </si>
-  <si>
     <t>F60-F69</t>
   </si>
   <si>
-    <t>Умственная отсталость  (1)</t>
-  </si>
-  <si>
     <t>F70-F79</t>
   </si>
   <si>
-    <t>Нарушения психологического развития  (1)</t>
-  </si>
-  <si>
     <t>F80-F89</t>
   </si>
   <si>
-    <t>Системные атрофии, поражающие преимущественно центральную нервную систему  (1)</t>
-  </si>
-  <si>
     <t>G10-G13</t>
   </si>
   <si>
-    <t>Экстрапирамидные и другие двигательные нарушения  (2)</t>
-  </si>
-  <si>
     <t>G20-G26</t>
   </si>
   <si>
-    <t>Другие дегенеративные болезни нервной системы  (1)</t>
-  </si>
-  <si>
     <t>G30-G32</t>
   </si>
   <si>
-    <t>Демиелинизирующие болезни центральной нервной системы  (1)</t>
-  </si>
-  <si>
     <t>G35-G37</t>
   </si>
   <si>
-    <t>Эпизодические и пароксизмальные расстройства  (6)</t>
-  </si>
-  <si>
     <t>G40-G47</t>
   </si>
   <si>
-    <t>Поражения отдельных нервов, нервных корешков и сплетений  (5)</t>
-  </si>
-  <si>
     <t>G50-G59</t>
   </si>
   <si>
-    <t>Полиневропатии и другие поражения периферической нервной системы  (2)</t>
-  </si>
-  <si>
     <t>G60-G64</t>
   </si>
   <si>
-    <t>Церебральный паралич и другие паралитические синдромы  (2)</t>
-  </si>
-  <si>
     <t>G80-G83</t>
   </si>
   <si>
-    <t>Другие нарушения нервной системы  (3)</t>
-  </si>
-  <si>
     <t>G90-G99</t>
   </si>
   <si>
-    <t>Осложнения, связанные преимущественно с послеродовым периодом (o85-o92)  (7)</t>
-  </si>
-  <si>
     <t>O85-O92</t>
   </si>
   <si>
-    <t>Родоразрешение  (6)</t>
-  </si>
-  <si>
     <t>O80-O84</t>
   </si>
   <si>
-    <t>Осложнения родов и родоразрешения  (15)</t>
-  </si>
-  <si>
     <t>O60-O75</t>
   </si>
   <si>
-    <t>Медицинская помощь матери в связи с состоянием плода, амниотической полости и возможными трудностями родоразрешения  (19)</t>
-  </si>
-  <si>
     <t>O30-O48</t>
   </si>
   <si>
-    <t>Другие болезни матери, связанные преимущественно с беременностью  (9)</t>
-  </si>
-  <si>
     <t>O20-O29</t>
   </si>
   <si>
-    <t>Болезни конъюнктивы  (1)</t>
-  </si>
-  <si>
     <t>H10-H13</t>
   </si>
   <si>
-    <t>Болезни склеры, роговицы, радужной оболочки и цилиарного тела  (2)</t>
-  </si>
-  <si>
     <t>H15-H22</t>
   </si>
   <si>
-    <t>Болезни хрусталика  (2)</t>
-  </si>
-  <si>
     <t>H25-H28</t>
   </si>
   <si>
-    <t>Болезни сосудистой оболочки и сетчатки  (7)</t>
-  </si>
-  <si>
     <t>H30-H36</t>
   </si>
   <si>
-    <t>Отеки, протеинурия и гипертензивные расстройства во время беременности, родов и в послеродовом периоде  (1)</t>
-  </si>
-  <si>
     <t>O10-O16</t>
   </si>
   <si>
-    <t>Беременность с абортивным исходом  (4)</t>
-  </si>
-  <si>
     <t>O00-O08</t>
   </si>
   <si>
-    <t>Нарушения мочеполовой системы после медицинских процедур, не классифицированные в других рубриках  (2)</t>
-  </si>
-  <si>
     <t>N99</t>
   </si>
   <si>
-    <t>Невоспалительные болезни женских половых органов  (19)</t>
-  </si>
-  <si>
     <t>N80-N98</t>
   </si>
   <si>
-    <t>Воспалительные болезни женских тазовых органов  (2)</t>
-  </si>
-  <si>
     <t>N70-N77</t>
   </si>
   <si>
-    <t>Болезни молочной железы  (2)</t>
-  </si>
-  <si>
     <t>N60-N64</t>
   </si>
   <si>
-    <t>Болезни мужских половых органов  (4)</t>
-  </si>
-  <si>
     <t>N40-N51</t>
   </si>
   <si>
-    <t>Другие болезни мочевой системы  (7)</t>
-  </si>
-  <si>
     <t>N30-N39</t>
   </si>
   <si>
-    <t>Другие болезни почки и мочеточника  (2)</t>
-  </si>
-  <si>
     <t>N25-N29</t>
   </si>
   <si>
-    <t>Мочекаменная болезнь  (3)</t>
-  </si>
-  <si>
     <t>N20-N23</t>
   </si>
   <si>
-    <t>Глаукома  (5)</t>
-  </si>
-  <si>
     <t>H40-H42</t>
   </si>
   <si>
-    <t>Болезни стекловидного тела и глазного яблока  (3)</t>
-  </si>
-  <si>
     <t>H43-H45</t>
   </si>
   <si>
-    <t>Болезни мышц глаза, нарушения содружественного движения глаз, аккомодации и рефракции  (3)</t>
-  </si>
-  <si>
     <t>H49-H52</t>
   </si>
   <si>
-    <t>Болезни наружного уха  (2)</t>
-  </si>
-  <si>
     <t>H60-H62</t>
   </si>
   <si>
-    <t>Болезни среднего уха и сосцевидного отростка  (3)</t>
-  </si>
-  <si>
     <t>H65-H75</t>
   </si>
   <si>
-    <t>Болезни внутреннего уха  (3)</t>
-  </si>
-  <si>
     <t>H80-H83</t>
   </si>
   <si>
-    <t>Почечная недостаточность  (4)</t>
-  </si>
-  <si>
     <t>N17-N19</t>
   </si>
   <si>
-    <t>Тубулоинтерстициальные болезни почек  (4)</t>
-  </si>
-  <si>
     <t>N10-N16</t>
   </si>
   <si>
-    <t>Гломерулярные болезни  (3)</t>
-  </si>
-  <si>
     <t>N00-N08</t>
   </si>
   <si>
-    <t>Другие нарушения костно-мышечной системы и соединительной ткани  (2)</t>
-  </si>
-  <si>
     <t>M95-M99</t>
   </si>
   <si>
-    <t>Остеопатии и хондропатии  (5)</t>
-  </si>
-  <si>
     <t>M80-M94</t>
   </si>
   <si>
-    <t>Болезни мягких тканей  (1)</t>
-  </si>
-  <si>
     <t>M60-M79</t>
   </si>
   <si>
-    <t>Дорсопатии  (10)</t>
-  </si>
-  <si>
     <t>M40-M54</t>
   </si>
   <si>
-    <t>Системные поражения соединительной ткани  (2)</t>
-  </si>
-  <si>
     <t>M30-M36</t>
   </si>
   <si>
-    <t>Артропатии  (12)</t>
-  </si>
-  <si>
     <t>M00-M25</t>
   </si>
   <si>
-    <t>Другие болезни кожи и подкожной клетчатки  (2)</t>
-  </si>
-  <si>
     <t>L80-L99</t>
   </si>
   <si>
-    <t>Болезни придатков кожи  (7)</t>
-  </si>
-  <si>
     <t>L60-L75</t>
   </si>
   <si>
-    <t>Болезни кожи и подкожной клетчатки, связанные с воздействием излучения  (2)</t>
-  </si>
-  <si>
     <t>L55-L59</t>
   </si>
   <si>
-    <t>Крапивница и эритема  (2)</t>
-  </si>
-  <si>
     <t>L50-L54</t>
   </si>
   <si>
-    <t>Папулосквамозные нарушения  (2)</t>
-  </si>
-  <si>
     <t>L40-L45</t>
   </si>
   <si>
-    <t>Другие болезни уха  (2)</t>
-  </si>
-  <si>
     <t>H90-H95</t>
   </si>
   <si>
-    <t>Хронические ревматические болезни сердца  (2)</t>
-  </si>
-  <si>
     <t>I05-I09</t>
   </si>
   <si>
-    <t>Болезни, характеризующиеся повышенным кровяным давлением  (1)</t>
-  </si>
-  <si>
     <t>I10-I15</t>
   </si>
   <si>
-    <t>Ишемическая болезнь сердца  (3)</t>
-  </si>
-  <si>
     <t>I20-I25</t>
   </si>
   <si>
-    <t>Легочное сердце и нарушения легочного кровообращения  (5)</t>
-  </si>
-  <si>
     <t>I26-I28</t>
   </si>
   <si>
-    <t>Другие болезни сердца  (12)</t>
-  </si>
-  <si>
     <t>I30-I52</t>
   </si>
   <si>
-    <t>Цереброваскулярные болезни  (3)</t>
-  </si>
-  <si>
     <t>I60-I69</t>
   </si>
   <si>
-    <t>Болезни артерий, артериол и капилляров  (5)</t>
-  </si>
-  <si>
     <t>I70-I79</t>
   </si>
   <si>
-    <t>Дерматит и экзема  (4)</t>
-  </si>
-  <si>
     <t>L20-L30</t>
   </si>
   <si>
-    <t>Буллезные нарушения  (3)</t>
-  </si>
-  <si>
     <t>L10-L14</t>
   </si>
   <si>
-    <t>Инфекции кожи и подкожной клетчатки  (3)</t>
-  </si>
-  <si>
     <t>L00-L08</t>
   </si>
   <si>
-    <t>Другие болезни органов пищеварения  (2)</t>
-  </si>
-  <si>
     <t>K90-K93</t>
   </si>
   <si>
-    <t>Болезни желчного пузыря, желчевыводящих путей и поджелудочной железы  (4)</t>
-  </si>
-  <si>
     <t>K80-K87</t>
   </si>
   <si>
-    <t>Болезни печени  (4)</t>
-  </si>
-  <si>
     <t>K70-K77</t>
   </si>
   <si>
-    <t>Геморрой и перианальный венозный тромбоз  (1)</t>
-  </si>
-  <si>
     <t>K64</t>
   </si>
   <si>
-    <t>Другие болезни кишечника  (14)</t>
-  </si>
-  <si>
     <t>K55-K63</t>
   </si>
   <si>
-    <t>Неинфекционный энтерит и колит  (4)</t>
-  </si>
-  <si>
     <t>K50-K52</t>
   </si>
   <si>
-    <t>Грыжи  (5)</t>
-  </si>
-  <si>
     <t>K40-K46</t>
   </si>
   <si>
-    <t>Болезни аппендикса [червеобразного отростка]  (1)</t>
-  </si>
-  <si>
     <t>K35-K38</t>
   </si>
   <si>
-    <t>Болезни пищевода, желудка и двенадцатиперстной кишки  (3)</t>
-  </si>
-  <si>
     <t>K20-K31</t>
   </si>
   <si>
-    <t>Болезни полости рта, слюнных желез и челюстей  (3)</t>
-  </si>
-  <si>
     <t>K00-K14</t>
   </si>
   <si>
-    <t>Другие болезни органов дыхания  (1)</t>
-  </si>
-  <si>
     <t>J95-J99</t>
   </si>
   <si>
-    <t>Гнойные и некротические состояния нижних дыхательных путей  (1)</t>
-  </si>
-  <si>
     <t>J85-J86</t>
   </si>
   <si>
-    <t>Другие респираторные болезни, поражающие главным образом интерстициальную ткань  (3)</t>
-  </si>
-  <si>
     <t>J80-J84</t>
   </si>
   <si>
-    <t>Болезни легкого, вызванные внешними агентами  (1)</t>
-  </si>
-  <si>
     <t>J60-J70</t>
   </si>
   <si>
-    <t>Хронические болезни нижних дыхательных путей  (5)</t>
-  </si>
-  <si>
     <t>J40-J47</t>
   </si>
   <si>
-    <t>Другие болезни верхних дыхательных путей  (9)</t>
-  </si>
-  <si>
     <t>J30-J39</t>
   </si>
   <si>
-    <t>Другие острые респираторные инфекции нижних дыхательных путей  (2)</t>
-  </si>
-  <si>
     <t>J20-J22</t>
   </si>
   <si>
-    <t>Грипп и пневмония  (3)</t>
-  </si>
-  <si>
     <t>J10-J18</t>
   </si>
   <si>
-    <t>Грипп, вызванный определенным идентифицированным вирусом гриппа  (1)</t>
-  </si>
-  <si>
     <t>J09</t>
   </si>
   <si>
-    <t>Острые респираторные инфекции верхних дыхательных путей  (5)</t>
-  </si>
-  <si>
     <t>J00-J06</t>
   </si>
   <si>
-    <t>Другие и неуточненные болезни системы кровообращения  (3)</t>
-  </si>
-  <si>
     <t>I95-I99</t>
   </si>
   <si>
-    <t>Болезни вен, лимфатических сосудов и лимфатических узлов, не классифицированные в других рубриках  (5)</t>
-  </si>
-  <si>
     <t>I80-I89</t>
+  </si>
+  <si>
+    <t>Другие болезни, вызываемые хламидиями</t>
+  </si>
+  <si>
+    <t>Термические и химические ожоги</t>
+  </si>
+  <si>
+    <t>Последствия проникновения инородного тела через естественные отверстия</t>
+  </si>
+  <si>
+    <t>Травмы неуточненной части туловища, конечности или области тела</t>
+  </si>
+  <si>
+    <t>Травмы, захватывающие несколько областей тела</t>
+  </si>
+  <si>
+    <t>Травмы области голеностопного сустава и стопы</t>
+  </si>
+  <si>
+    <t>Травмы колена и голени</t>
+  </si>
+  <si>
+    <t>Травмы области тазобедренного сустава и бедра</t>
+  </si>
+  <si>
+    <t>Травмы запястья и кисти</t>
+  </si>
+  <si>
+    <t>Травмы локтя и предплечья</t>
+  </si>
+  <si>
+    <t>Травмы плечевого пояса и плеча</t>
+  </si>
+  <si>
+    <t>Травмы живота, нижней части спины, поясничного отдела позвоночника и таза</t>
+  </si>
+  <si>
+    <t>Травмы грудной клетки</t>
+  </si>
+  <si>
+    <t>Травмы шеи</t>
+  </si>
+  <si>
+    <t>Травмы головы</t>
+  </si>
+  <si>
+    <t>Отклонения от нормы, выявленные при исследовании крови, при отсутствии установленного диагноза</t>
+  </si>
+  <si>
+    <t>Общие симптомы и признаки</t>
+  </si>
+  <si>
+    <t>Симптомы и признаки, относящиеся к мочевой системе</t>
+  </si>
+  <si>
+    <t>Симптомы и признаки, относящиеся к системе пищеварения и брюшной полости</t>
+  </si>
+  <si>
+    <t>Симптомы и признаки, относящиеся к системам кровообращения и дыхания</t>
+  </si>
+  <si>
+    <t>Другие врожденные аномалии [пороки развития]</t>
+  </si>
+  <si>
+    <t>Врожденные аномалии [пороки развития] и деформации костно-мышечной системы</t>
+  </si>
+  <si>
+    <t>Врожденные аномалии [пороки развития] мочевой системы</t>
+  </si>
+  <si>
+    <t>Другие врожденные аномалии [пороки развития] органов пищеварения</t>
+  </si>
+  <si>
+    <t>Врожденные аномалии [пороки развития] системы кровообращения</t>
+  </si>
+  <si>
+    <t>Врожденные аномалии [пороки развития] глаза, уха, лица и шеи</t>
+  </si>
+  <si>
+    <t>Другие нарушения, возникающие в перинатальном периоде</t>
+  </si>
+  <si>
+    <t>Геморрагические и гематологические нарушения у плода и новорожденного</t>
+  </si>
+  <si>
+    <t>Инфекционные болезни, специфичные для перинатального периода</t>
+  </si>
+  <si>
+    <t>Дыхательные и сердечно-сосудистые нарушения, характерные для перинатального периода</t>
+  </si>
+  <si>
+    <t>Расстройства, связанные с продолжительностью беременности и ростом плода</t>
+  </si>
+  <si>
+    <t>Другие акушерские состояния, не классифицированные в других рубриках</t>
+  </si>
+  <si>
+    <t>Осложнения, связанные преимущественно с послеродовым периодом</t>
+  </si>
+  <si>
+    <t>Родоразрешение</t>
+  </si>
+  <si>
+    <t>Осложнения родов и родоразрешения</t>
+  </si>
+  <si>
+    <t>Медицинская помощь матери в связи с состоянием плода, амниотической полости и возможными трудностями родоразрешения</t>
+  </si>
+  <si>
+    <t>Вирусные инфекции центральной нервной системы</t>
+  </si>
+  <si>
+    <t>Вирусные лихорадки, передаваемые членистоногими, и вирусные геморрагические лихорадки</t>
+  </si>
+  <si>
+    <t>Вирусные инфекции, характеризующиеся поражениями кожи и слизистых оболочек</t>
+  </si>
+  <si>
+    <t>Вирусный гепатит</t>
+  </si>
+  <si>
+    <t>Болезнь, вызванная вирусом иммунодефицита человека [вич]</t>
+  </si>
+  <si>
+    <t>Другие вирусные болезни</t>
+  </si>
+  <si>
+    <t>Микозы</t>
+  </si>
+  <si>
+    <t>Гельминтозы</t>
+  </si>
+  <si>
+    <t>Последствия инфекционных и паразитарных болезней</t>
+  </si>
+  <si>
+    <t>Бактериальные, вирусные и другие инфекционные агенты</t>
+  </si>
+  <si>
+    <t>Злокачественные новообразования</t>
+  </si>
+  <si>
+    <t>Новообразования in situ</t>
+  </si>
+  <si>
+    <t>Доброкачественные новообразования</t>
+  </si>
+  <si>
+    <t>Новообразования неопределенного или неизвестного характера</t>
+  </si>
+  <si>
+    <t>Анемии, связанные с питанием</t>
+  </si>
+  <si>
+    <t>Гемолитические анемии</t>
+  </si>
+  <si>
+    <t>Апластические и другие анемии</t>
+  </si>
+  <si>
+    <t>Нарушения свертываемости крови, пурпура и другие геморрагические состояния</t>
+  </si>
+  <si>
+    <t>Другие болезни матери, связанные преимущественно с беременностью</t>
+  </si>
+  <si>
+    <t>Отеки, протеинурия и гипертензивные расстройства во время беременности, родов и в послеродовом периоде</t>
+  </si>
+  <si>
+    <t>Беременность с абортивным исходом</t>
+  </si>
+  <si>
+    <t>Нарушения мочеполовой системы после медицинских процедур, не классифицированные в других рубриках</t>
+  </si>
+  <si>
+    <t>Невоспалительные болезни женских половых органов</t>
+  </si>
+  <si>
+    <t>Воспалительные болезни женских тазовых органов</t>
+  </si>
+  <si>
+    <t>Болезни молочной железы</t>
+  </si>
+  <si>
+    <t>Болезни мужских половых органов</t>
+  </si>
+  <si>
+    <t>Другие болезни мочевой системы</t>
+  </si>
+  <si>
+    <t>Другие болезни почки и мочеточника</t>
+  </si>
+  <si>
+    <t>Мочекаменная болезнь</t>
+  </si>
+  <si>
+    <t>Почечная недостаточность</t>
+  </si>
+  <si>
+    <t>Тубулоинтерстициальные болезни почек</t>
+  </si>
+  <si>
+    <t>Гломерулярные болезни</t>
+  </si>
+  <si>
+    <t>Другие нарушения костно-мышечной системы и соединительной ткани</t>
+  </si>
+  <si>
+    <t>Остеопатии и хондропатии</t>
+  </si>
+  <si>
+    <t>Болезни мягких тканей</t>
+  </si>
+  <si>
+    <t>Дорсопатии</t>
+  </si>
+  <si>
+    <t>Системные поражения соединительной ткани</t>
+  </si>
+  <si>
+    <t>Артропатии</t>
+  </si>
+  <si>
+    <t>Другие болезни кожи и подкожной клетчатки</t>
+  </si>
+  <si>
+    <t>Болезни придатков кожи</t>
+  </si>
+  <si>
+    <t>Болезни кожи и подкожной клетчатки, связанные с воздействием излучения</t>
+  </si>
+  <si>
+    <t>Крапивница и эритема</t>
+  </si>
+  <si>
+    <t>Папулосквамозные нарушения</t>
+  </si>
+  <si>
+    <t>Дерматит и экзема</t>
+  </si>
+  <si>
+    <t>Буллезные нарушения</t>
+  </si>
+  <si>
+    <t>Инфекции кожи и подкожной клетчатки</t>
+  </si>
+  <si>
+    <t>Другие болезни органов пищеварения</t>
+  </si>
+  <si>
+    <t>Болезни желчного пузыря, желчевыводящих путей и поджелудочной железы</t>
+  </si>
+  <si>
+    <t>Болезни печени</t>
+  </si>
+  <si>
+    <t>Геморрой и перианальный венозный тромбоз</t>
+  </si>
+  <si>
+    <t>Другие болезни кишечника</t>
+  </si>
+  <si>
+    <t>Неинфекционный энтерит и колит</t>
+  </si>
+  <si>
+    <t>Грыжи</t>
+  </si>
+  <si>
+    <t>Болезни аппендикса [червеобразного отростка]</t>
+  </si>
+  <si>
+    <t>Болезни пищевода, желудка и двенадцатиперстной кишки</t>
+  </si>
+  <si>
+    <t>Болезни полости рта, слюнных желез и челюстей</t>
+  </si>
+  <si>
+    <t>Другие болезни органов дыхания</t>
+  </si>
+  <si>
+    <t>Гнойные и некротические состояния нижних дыхательных путей</t>
+  </si>
+  <si>
+    <t>Другие респираторные болезни, поражающие главным образом интерстициальную ткань</t>
+  </si>
+  <si>
+    <t>Болезни легкого, вызванные внешними агентами</t>
+  </si>
+  <si>
+    <t>Хронические болезни нижних дыхательных путей</t>
+  </si>
+  <si>
+    <t>Другие болезни верхних дыхательных путей</t>
+  </si>
+  <si>
+    <t>Другие острые респираторные инфекции нижних дыхательных путей</t>
+  </si>
+  <si>
+    <t>Грипп и пневмония</t>
+  </si>
+  <si>
+    <t>Грипп, вызванный определенным идентифицированным вирусом гриппа</t>
+  </si>
+  <si>
+    <t>Острые респираторные инфекции верхних дыхательных путей</t>
+  </si>
+  <si>
+    <t>Другие и неуточненные болезни системы кровообращения</t>
+  </si>
+  <si>
+    <t>Болезни вен, лимфатических сосудов и лимфатических узлов, не классифицированные в других рубриках</t>
+  </si>
+  <si>
+    <t>Болезни артерий, артериол и капилляров</t>
+  </si>
+  <si>
+    <t>Цереброваскулярные болезни</t>
+  </si>
+  <si>
+    <t>Другие болезни сердца</t>
+  </si>
+  <si>
+    <t>Легочное сердце и нарушения легочного кровообращения</t>
+  </si>
+  <si>
+    <t>Ишемическая болезнь сердца</t>
+  </si>
+  <si>
+    <t>Болезни, характеризующиеся повышенным кровяным давлением</t>
+  </si>
+  <si>
+    <t>Хронические ревматические болезни сердца</t>
+  </si>
+  <si>
+    <t>Другие болезни уха</t>
+  </si>
+  <si>
+    <t>Болезни внутреннего уха</t>
+  </si>
+  <si>
+    <t>Болезни среднего уха и сосцевидного отростка</t>
+  </si>
+  <si>
+    <t>Болезни наружного уха</t>
+  </si>
+  <si>
+    <t>Болезни мышц глаза, нарушения содружественного движения глаз, аккомодации и рефракции</t>
+  </si>
+  <si>
+    <t>Болезни стекловидного тела и глазного яблока</t>
+  </si>
+  <si>
+    <t>Глаукома</t>
+  </si>
+  <si>
+    <t>Болезни сосудистой оболочки и сетчатки</t>
+  </si>
+  <si>
+    <t>Болезни хрусталика</t>
+  </si>
+  <si>
+    <t>Болезни склеры, роговицы, радужной оболочки и цилиарного тела</t>
+  </si>
+  <si>
+    <t>Болезни конъюнктивы</t>
+  </si>
+  <si>
+    <t>Другие нарушения нервной системы</t>
+  </si>
+  <si>
+    <t>Церебральный паралич и другие паралитические синдромы</t>
+  </si>
+  <si>
+    <t>Полиневропатии и другие поражения периферической нервной системы</t>
+  </si>
+  <si>
+    <t>Поражения отдельных нервов, нервных корешков и сплетений</t>
+  </si>
+  <si>
+    <t>Эпизодические и пароксизмальные расстройства</t>
+  </si>
+  <si>
+    <t>Демиелинизирующие болезни центральной нервной системы</t>
+  </si>
+  <si>
+    <t>Другие дегенеративные болезни нервной системы</t>
+  </si>
+  <si>
+    <t>Экстрапирамидные и другие двигательные нарушения</t>
+  </si>
+  <si>
+    <t>Системные атрофии, поражающие преимущественно центральную нервную систему</t>
+  </si>
+  <si>
+    <t>Нарушения психологического развития</t>
+  </si>
+  <si>
+    <t>Умственная отсталость</t>
+  </si>
+  <si>
+    <t>Расстройства личности и поведения в зрелом возрасте</t>
+  </si>
+  <si>
+    <t>Поведенческие синдромы, связанные с физиологическими нарушениями и физическими факторами</t>
+  </si>
+  <si>
+    <t>Невротические, связанные со стрессом и соматоформные расстройства</t>
+  </si>
+  <si>
+    <t>Расстройства настроения [аффективные расстройства]</t>
+  </si>
+  <si>
+    <t>Шизофрения, шизотипические состояния и бредовые расстройства</t>
+  </si>
+  <si>
+    <t>Психические расстройства и расстройства поведения, связанные с употреблением психоактивных веществ</t>
+  </si>
+  <si>
+    <t>Органические, включая симптоматические, психические расстройства</t>
+  </si>
+  <si>
+    <t>Нарушения обмена веществ</t>
+  </si>
+  <si>
+    <t>Ожирение и другие виды избыточности питания</t>
+  </si>
+  <si>
+    <t>Другие виды недостаточности питания</t>
+  </si>
+  <si>
+    <t>Недостаточность питания</t>
+  </si>
+  <si>
+    <t>Нарушения других эндокринных желез</t>
+  </si>
+  <si>
+    <t>Сахарный диабет</t>
+  </si>
+  <si>
+    <t>Болезни щитовидной железы</t>
+  </si>
+  <si>
+    <t>Отдельные нарушения, вовлекающие иммунный механизм</t>
+  </si>
+  <si>
+    <t>Другие болезни крови и кроветворных органов</t>
   </si>
 </sst>
 </file>
@@ -1495,743 +1495,743 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>78</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>80</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>82</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>84</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>86</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>88</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>66</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>90</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>93</v>
+        <v>67</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>92</v>
+        <v>233</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>94</v>
+        <v>234</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>96</v>
+        <v>235</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>98</v>
+        <v>236</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>100</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>103</v>
+        <v>72</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>102</v>
+        <v>238</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>105</v>
+        <v>73</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>104</v>
+        <v>239</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>106</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>108</v>
+        <v>241</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>110</v>
+        <v>242</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>112</v>
+        <v>243</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>115</v>
+        <v>78</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>114</v>
+        <v>244</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>116</v>
+        <v>339</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>118</v>
+        <v>338</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>147</v>
+        <v>94</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>146</v>
+        <v>337</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>149</v>
+        <v>95</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>148</v>
+        <v>336</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>151</v>
+        <v>96</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>150</v>
+        <v>335</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" t="s">
-        <v>153</v>
+        <v>97</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>152</v>
+        <v>334</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>155</v>
+        <v>98</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>154</v>
+        <v>333</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>157</v>
+        <v>99</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>156</v>
+        <v>332</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>159</v>
+        <v>100</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>158</v>
+        <v>331</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>161</v>
+        <v>101</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>160</v>
+        <v>330</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>163</v>
+        <v>102</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>162</v>
+        <v>329</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
-        <v>165</v>
+        <v>103</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>164</v>
+        <v>328</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>167</v>
+        <v>104</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>166</v>
+        <v>327</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>169</v>
+        <v>105</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>168</v>
+        <v>326</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>171</v>
+        <v>106</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>170</v>
+        <v>325</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>173</v>
+        <v>107</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>172</v>
+        <v>324</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>175</v>
+        <v>108</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>174</v>
+        <v>323</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" t="s">
-        <v>177</v>
+        <v>109</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>176</v>
+        <v>322</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" t="s">
-        <v>179</v>
+        <v>110</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>178</v>
+        <v>321</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45" t="s">
-        <v>181</v>
+        <v>111</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>180</v>
+        <v>320</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>183</v>
+        <v>112</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>182</v>
+        <v>319</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" t="s">
-        <v>185</v>
+        <v>113</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>184</v>
+        <v>318</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" t="s">
-        <v>187</v>
+        <v>114</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>186</v>
+        <v>317</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>189</v>
+        <v>115</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>188</v>
+        <v>316</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>191</v>
+        <v>116</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>190</v>
+        <v>315</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>193</v>
+        <v>117</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>192</v>
+        <v>314</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
-        <v>195</v>
+        <v>118</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>194</v>
+        <v>313</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
-        <v>207</v>
+        <v>124</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>206</v>
+        <v>312</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" t="s">
-        <v>209</v>
+        <v>125</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>208</v>
+        <v>311</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" t="s">
-        <v>211</v>
+        <v>126</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>210</v>
+        <v>310</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" t="s">
-        <v>213</v>
+        <v>127</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>212</v>
+        <v>309</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" t="s">
-        <v>235</v>
+        <v>138</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>234</v>
+        <v>308</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58" t="s">
-        <v>237</v>
+        <v>139</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>236</v>
+        <v>307</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" t="s">
-        <v>239</v>
+        <v>140</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>238</v>
+        <v>306</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60" t="s">
-        <v>241</v>
+        <v>141</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>240</v>
+        <v>305</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" t="s">
-        <v>243</v>
+        <v>142</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>242</v>
+        <v>304</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" t="s">
-        <v>245</v>
+        <v>143</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>244</v>
+        <v>303</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" t="s">
-        <v>275</v>
+        <v>158</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>274</v>
+        <v>302</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" t="s">
-        <v>277</v>
+        <v>159</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>276</v>
+        <v>301</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65" t="s">
-        <v>279</v>
+        <v>160</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>278</v>
+        <v>300</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" t="s">
-        <v>281</v>
+        <v>161</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>280</v>
+        <v>299</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67" t="s">
-        <v>283</v>
+        <v>162</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>282</v>
+        <v>298</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68" t="s">
-        <v>285</v>
+        <v>163</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69" t="s">
-        <v>287</v>
+        <v>164</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70" t="s">
-        <v>289</v>
+        <v>165</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="16.5" customHeight="1">
       <c r="A71" t="s">
-        <v>339</v>
+        <v>190</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>338</v>
+        <v>294</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72" t="s">
-        <v>337</v>
+        <v>189</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>336</v>
+        <v>293</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73" t="s">
-        <v>335</v>
+        <v>188</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>334</v>
+        <v>292</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74" t="s">
-        <v>333</v>
+        <v>187</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>332</v>
+        <v>291</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75" t="s">
-        <v>331</v>
+        <v>186</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>330</v>
+        <v>290</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76" t="s">
-        <v>329</v>
+        <v>185</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>328</v>
+        <v>289</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77" t="s">
-        <v>327</v>
+        <v>184</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>326</v>
+        <v>288</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78" t="s">
-        <v>325</v>
+        <v>183</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>324</v>
+        <v>287</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79" t="s">
-        <v>323</v>
+        <v>182</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>322</v>
+        <v>286</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80" t="s">
-        <v>321</v>
+        <v>181</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>320</v>
+        <v>285</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81" t="s">
-        <v>319</v>
+        <v>180</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>318</v>
+        <v>284</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82" t="s">
-        <v>317</v>
+        <v>179</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>316</v>
+        <v>283</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83" t="s">
-        <v>315</v>
+        <v>178</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>314</v>
+        <v>282</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84" t="s">
-        <v>313</v>
+        <v>177</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>312</v>
+        <v>281</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85" t="s">
-        <v>311</v>
+        <v>176</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>310</v>
+        <v>280</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86" t="s">
-        <v>309</v>
+        <v>175</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>308</v>
+        <v>279</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87" t="s">
-        <v>307</v>
+        <v>174</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>306</v>
+        <v>278</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88" t="s">
-        <v>305</v>
+        <v>173</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>304</v>
+        <v>277</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89" t="s">
-        <v>303</v>
+        <v>172</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>302</v>
+        <v>276</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90" t="s">
-        <v>301</v>
+        <v>171</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>300</v>
+        <v>275</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91" t="s">
-        <v>299</v>
+        <v>170</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>298</v>
+        <v>274</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92" t="s">
-        <v>297</v>
+        <v>169</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93" t="s">
-        <v>295</v>
+        <v>168</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>294</v>
+        <v>272</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94" t="s">
-        <v>293</v>
+        <v>167</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>292</v>
+        <v>271</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95" t="s">
-        <v>291</v>
+        <v>166</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96" t="s">
-        <v>273</v>
+        <v>157</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97" t="s">
-        <v>271</v>
+        <v>156</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98" t="s">
-        <v>269</v>
+        <v>155</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99" t="s">
-        <v>267</v>
+        <v>154</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>266</v>
@@ -2239,450 +2239,450 @@
     </row>
     <row r="100" spans="1:2">
       <c r="A100" t="s">
+        <v>153</v>
+      </c>
+      <c r="B100" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101" t="s">
-        <v>263</v>
+        <v>152</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="102" spans="1:2">
       <c r="A102" t="s">
-        <v>261</v>
+        <v>151</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="103" spans="1:2">
       <c r="A103" t="s">
-        <v>259</v>
+        <v>150</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="104" spans="1:2">
       <c r="A104" t="s">
-        <v>257</v>
+        <v>149</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="105" spans="1:2">
       <c r="A105" t="s">
-        <v>255</v>
+        <v>148</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
     </row>
     <row r="106" spans="1:2">
       <c r="A106" t="s">
-        <v>253</v>
+        <v>147</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="107" spans="1:2">
       <c r="A107" t="s">
-        <v>251</v>
+        <v>146</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
     </row>
     <row r="108" spans="1:2">
       <c r="A108" t="s">
-        <v>249</v>
+        <v>145</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="109" spans="1:2">
       <c r="A109" t="s">
-        <v>247</v>
+        <v>144</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
     </row>
     <row r="110" spans="1:2">
       <c r="A110" t="s">
-        <v>233</v>
+        <v>137</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>232</v>
+        <v>255</v>
       </c>
     </row>
     <row r="111" spans="1:2">
       <c r="A111" t="s">
-        <v>231</v>
+        <v>136</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>230</v>
+        <v>254</v>
       </c>
     </row>
     <row r="112" spans="1:2">
       <c r="A112" t="s">
-        <v>229</v>
+        <v>135</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>228</v>
+        <v>253</v>
       </c>
     </row>
     <row r="113" spans="1:2">
       <c r="A113" t="s">
-        <v>227</v>
+        <v>134</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>226</v>
+        <v>252</v>
       </c>
     </row>
     <row r="114" spans="1:2">
       <c r="A114" t="s">
-        <v>225</v>
+        <v>133</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>224</v>
+        <v>251</v>
       </c>
     </row>
     <row r="115" spans="1:2">
       <c r="A115" t="s">
-        <v>223</v>
+        <v>132</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>222</v>
+        <v>250</v>
       </c>
     </row>
     <row r="116" spans="1:2">
       <c r="A116" t="s">
-        <v>221</v>
+        <v>131</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>220</v>
+        <v>249</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="21.75" customHeight="1">
       <c r="A117" t="s">
-        <v>219</v>
+        <v>130</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>218</v>
+        <v>248</v>
       </c>
     </row>
     <row r="118" spans="1:2">
       <c r="A118" t="s">
-        <v>217</v>
+        <v>129</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" ht="30">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
       <c r="A119" t="s">
-        <v>215</v>
+        <v>128</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>214</v>
+        <v>246</v>
       </c>
     </row>
     <row r="120" spans="1:2">
       <c r="A120" t="s">
-        <v>205</v>
+        <v>123</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>204</v>
+        <v>245</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="30">
       <c r="A121" t="s">
-        <v>203</v>
+        <v>122</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>202</v>
+        <v>226</v>
       </c>
     </row>
     <row r="122" spans="1:2">
       <c r="A122" t="s">
-        <v>201</v>
+        <v>121</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>200</v>
+        <v>225</v>
       </c>
     </row>
     <row r="123" spans="1:2">
       <c r="A123" t="s">
-        <v>199</v>
+        <v>120</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
     </row>
     <row r="124" spans="1:2">
       <c r="A124" t="s">
-        <v>197</v>
+        <v>119</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>196</v>
+        <v>223</v>
       </c>
     </row>
     <row r="125" spans="1:2">
       <c r="A125" t="s">
-        <v>145</v>
+        <v>93</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>144</v>
+        <v>222</v>
       </c>
     </row>
     <row r="126" spans="1:2">
       <c r="A126" t="s">
-        <v>143</v>
+        <v>92</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>142</v>
+        <v>221</v>
       </c>
     </row>
     <row r="127" spans="1:2">
       <c r="A127" t="s">
-        <v>141</v>
+        <v>91</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>140</v>
+        <v>220</v>
       </c>
     </row>
     <row r="128" spans="1:2">
       <c r="A128" t="s">
-        <v>139</v>
+        <v>90</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>138</v>
+        <v>219</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="A129" t="s">
-        <v>137</v>
+        <v>89</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>136</v>
+        <v>218</v>
       </c>
     </row>
     <row r="130" spans="1:2">
       <c r="A130" t="s">
-        <v>135</v>
+        <v>88</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>134</v>
+        <v>217</v>
       </c>
     </row>
     <row r="131" spans="1:2">
       <c r="A131" t="s">
-        <v>133</v>
+        <v>87</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>132</v>
+        <v>216</v>
       </c>
     </row>
     <row r="132" spans="1:2">
       <c r="A132" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>130</v>
+        <v>215</v>
       </c>
     </row>
     <row r="133" spans="1:2">
       <c r="A133" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>128</v>
+        <v>214</v>
       </c>
     </row>
     <row r="134" spans="1:2">
       <c r="A134" t="s">
-        <v>127</v>
+        <v>84</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>126</v>
+        <v>213</v>
       </c>
     </row>
     <row r="135" spans="1:2">
       <c r="A135" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>124</v>
+        <v>212</v>
       </c>
     </row>
     <row r="136" spans="1:2">
       <c r="A136" t="s">
-        <v>121</v>
+        <v>81</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>120</v>
+        <v>211</v>
       </c>
     </row>
     <row r="137" spans="1:2">
       <c r="A137" t="s">
-        <v>123</v>
+        <v>82</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>122</v>
+        <v>210</v>
       </c>
     </row>
     <row r="138" spans="1:2">
       <c r="A138" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>76</v>
+        <v>209</v>
       </c>
     </row>
     <row r="139" spans="1:2">
       <c r="A139" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>74</v>
+        <v>208</v>
       </c>
     </row>
     <row r="140" spans="1:2">
       <c r="A140" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>72</v>
+        <v>207</v>
       </c>
     </row>
     <row r="141" spans="1:2">
       <c r="A141" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>70</v>
+        <v>206</v>
       </c>
     </row>
     <row r="142" spans="1:2">
       <c r="A142" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>68</v>
+        <v>205</v>
       </c>
     </row>
     <row r="143" spans="1:2">
       <c r="A143" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>66</v>
+        <v>204</v>
       </c>
     </row>
     <row r="144" spans="1:2">
       <c r="A144" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>64</v>
+        <v>203</v>
       </c>
     </row>
     <row r="145" spans="1:2">
       <c r="A145" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>62</v>
+        <v>202</v>
       </c>
     </row>
     <row r="146" spans="1:2">
       <c r="A146" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>60</v>
+        <v>201</v>
       </c>
     </row>
     <row r="147" spans="1:2">
       <c r="A147" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>58</v>
+        <v>200</v>
       </c>
     </row>
     <row r="148" spans="1:2">
       <c r="A148" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>56</v>
+        <v>199</v>
       </c>
     </row>
     <row r="149" spans="1:2">
       <c r="A149" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>54</v>
+        <v>198</v>
       </c>
     </row>
     <row r="150" spans="1:2">
       <c r="A150" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>52</v>
+        <v>197</v>
       </c>
     </row>
     <row r="151" spans="1:2">
       <c r="A151" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>50</v>
+        <v>196</v>
       </c>
     </row>
     <row r="152" spans="1:2">
       <c r="A152" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>48</v>
+        <v>195</v>
       </c>
     </row>
     <row r="153" spans="1:2">
       <c r="A153" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>46</v>
+        <v>194</v>
       </c>
     </row>
     <row r="154" spans="1:2">
       <c r="A154" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>44</v>
+        <v>193</v>
       </c>
     </row>
     <row r="155" spans="1:2">
       <c r="A155" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>42</v>
+        <v>192</v>
       </c>
     </row>
     <row r="156" spans="1:2">

</xml_diff>